<commit_message>
Adauga observatia saltbox parsel-app si findings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TkfYT2KFEgW3ePKEgphig
</commit_message>
<xml_diff>
--- a/Observatii.xlsx
+++ b/Observatii.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Observații</t>
   </si>
   <si>
-    <t xml:space="preserve">Completezi coloanele B (Pagina URL) și C (Comentariul meu), marcate cu galben. Coloana D (Findings) o completează Claude pe baza comentariului tău. Rândul 5 este un exemplu – îl poți șterge.</t>
+    <t xml:space="preserve">Completezi coloanele B (Pagina URL) și C (Comentariul meu), marcate cu galben. Coloana D (Findings) o completează Claude pe baza comentariului tău.</t>
   </si>
   <si>
     <t xml:space="preserve">Nr.</t>
@@ -44,13 +44,15 @@
     <t xml:space="preserve">Findings</t>
   </si>
   <si>
-    <t xml:space="preserve">https://example.com/contact</t>
+    <t xml:space="preserve">https://www.saltbox.com/services/parsel-app</t>
   </si>
   <si>
-    <t xml:space="preserve">Formularul de contact nu trimite mesajul.</t>
+    <t xml:space="preserve">dispare ce-overview_content-right la mobile landscape</t>
   </si>
   <si>
-    <t xml:space="preserve">(Exemplu) Butonul „Trimite” nu are acțiune setată; după click nu apare mesaj de succes sau eroare. Câmpul email nu are validare. Recomandare: verifică setările formularului și adaugă mesaje de confirmare.</t>
+    <t xml:space="preserve">CONFIRMAT. Div-ul are și clasa hide-mobile-landscape; regula din Global Styles @media (max-width:767px){.hide-mobile-landscape{display:none !important}} îl ascunde sub 767px. Efect: pe mobil hero-ul rămâne doar cu H1, fără text și fără butoanele Try Parsel / Login to Parsel. Nu e cauzat de interacțiuni IX2.
+FIX: în Webflow Designer scoate clasa hide-mobile-landscape de pe ce-overview_content-right (nu modifica regula globală, o mai folosesc alte 20 de elemente). Verifică la 767px și 479px că header15_content-wrapper trece pe o coloană.
+Alte probleme: imaginea din tab-ul vizibil implicit (header103) are loading=lazy, iar cea din tab-ul ascuns eager + fetchpriority=high (LCP); iconițele tag-icon au width/height=0.</t>
   </si>
 </sst>
 </file>
@@ -108,9 +110,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
       <sz val="10"/>
-      <color rgb="FF808080"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -192,12 +192,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -242,7 +246,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -262,14 +266,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF808080"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -541,494 +537,494 @@
   <dimension ref="A1:D54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+    <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <f aca="false">IF(B5="","",ROW()-4)</f>
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="str">
         <f aca="false">IF(B6="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="str">
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="str">
         <f aca="false">IF(B7="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="9"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="str">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="str">
         <f aca="false">IF(B8="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="str">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="str">
         <f aca="false">IF(B9="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="str">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="str">
         <f aca="false">IF(B10="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="str">
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="str">
         <f aca="false">IF(B11="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="str">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="str">
         <f aca="false">IF(B12="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="str">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="str">
         <f aca="false">IF(B13="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="str">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="str">
         <f aca="false">IF(B14="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="str">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="str">
         <f aca="false">IF(B15="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="str">
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="str">
         <f aca="false">IF(B16="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="str">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="str">
         <f aca="false">IF(B17="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="str">
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="str">
         <f aca="false">IF(B18="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="str">
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="str">
         <f aca="false">IF(B19="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="str">
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="str">
         <f aca="false">IF(B20="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="str">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="str">
         <f aca="false">IF(B21="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="str">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="str">
         <f aca="false">IF(B22="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="str">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="10"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="str">
         <f aca="false">IF(B23="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="str">
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="10"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="str">
         <f aca="false">IF(B24="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="str">
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="10"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="str">
         <f aca="false">IF(B25="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="str">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="str">
         <f aca="false">IF(B26="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="str">
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="10"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="str">
         <f aca="false">IF(B27="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="9"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="str">
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="str">
         <f aca="false">IF(B28="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="str">
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="str">
         <f aca="false">IF(B29="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="str">
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="str">
         <f aca="false">IF(B30="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="str">
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="10"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="str">
         <f aca="false">IF(B31="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="9"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="str">
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="str">
         <f aca="false">IF(B32="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="str">
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="str">
         <f aca="false">IF(B33="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="str">
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="str">
         <f aca="false">IF(B34="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="9"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="str">
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="10"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="str">
         <f aca="false">IF(B35="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="str">
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="10"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="str">
         <f aca="false">IF(B36="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="str">
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="10"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="str">
         <f aca="false">IF(B37="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="str">
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="10"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="str">
         <f aca="false">IF(B38="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="str">
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="10"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="str">
         <f aca="false">IF(B39="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="str">
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="10"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="str">
         <f aca="false">IF(B40="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="9"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="str">
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="10"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="str">
         <f aca="false">IF(B41="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="str">
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="str">
         <f aca="false">IF(B42="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="str">
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="10"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="str">
         <f aca="false">IF(B43="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="str">
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="10"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="str">
         <f aca="false">IF(B44="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="str">
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="10"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="str">
         <f aca="false">IF(B45="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="str">
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="10"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8" t="str">
         <f aca="false">IF(B46="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="str">
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="10"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="str">
         <f aca="false">IF(B47="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="str">
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="10"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="8" t="str">
         <f aca="false">IF(B48="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="str">
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="10"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="8" t="str">
         <f aca="false">IF(B49="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="str">
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="10"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="8" t="str">
         <f aca="false">IF(B50="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="str">
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="10"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8" t="str">
         <f aca="false">IF(B51="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="str">
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="10"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="8" t="str">
         <f aca="false">IF(B52="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="9"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="str">
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="10"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="str">
         <f aca="false">IF(B53="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="str">
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="10"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="8" t="str">
         <f aca="false">IF(B54="","",ROW()-4)</f>
         <v/>
       </c>
-      <c r="B54" s="8"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:D54"/>

</xml_diff>

<commit_message>
Adauga observatia saltbox blog-overview si findings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TkfYT2KFEgW3ePKEgphig
</commit_message>
<xml_diff>
--- a/Observatii.xlsx
+++ b/Observatii.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Observații</t>
   </si>
@@ -53,6 +53,17 @@
     <t xml:space="preserve">CONFIRMAT. Div-ul are și clasa hide-mobile-landscape; regula din Global Styles @media (max-width:767px){.hide-mobile-landscape{display:none !important}} îl ascunde sub 767px. Efect: pe mobil hero-ul rămâne doar cu H1, fără text și fără butoanele Try Parsel / Login to Parsel. Nu e cauzat de interacțiuni IX2.
 FIX: în Webflow Designer scoate clasa hide-mobile-landscape de pe ce-overview_content-right (nu modifica regula globală, o mai folosesc alte 20 de elemente). Verifică la 767px și 479px că header15_content-wrapper trece pe o coloană.
 Alte probleme: imaginea din tab-ul vizibil implicit (header103) are loading=lazy, iar cea din tab-ul ascuns eager + fetchpriority=high (LCP); iconițele tag-icon au width/height=0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.saltbox.com/resources/blog-overview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cardul mobile-blog-card se dubleaza la mobile si este hide la desk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARȚIAL CONFIRMAT. Dublarea e reală, dar vine din CMS, nu din CSS-ul cardului: articolul „Meet the three finalists for our $5,000 Atlanta small business grant” apare ca featured și ca item 6 în lista principală (.blog21_list), pe mobil ȘI pe desktop. Lista principală nu exclude articolul featured. Ascunderea mobile-blog-card pe desktop e intenționată (swap desktop/mobil: cardurile desktop au hide-mobile-landscape).
+FIX: Collection List Settings pe lista principală → filtru care exclude featured (ex. Featured is Off) sau Start at item 2 cu aceeași sortare. Clasa mobile-blog-card nu trebuie modificată.
+Alte probleme: fiecare card e de 2 ori în DOM (linkuri/imagini duplicate); cardul featured nu e afectat de filtrele de categorie; h4 pe desktop / h6 pe mobil, alt gol la imagini, linkuri „Read more” generice. Tableta (768–991px) neverificată.</t>
   </si>
 </sst>
 </file>
@@ -586,13 +597,19 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="str">
+      <c r="A6" s="5" t="n">
         <f aca="false">IF(B6="","",ROW()-4)</f>
-        <v/>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="10"/>
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="str">

</xml_diff>

<commit_message>
Adauga observatia saltbox member-stories (buton absolut)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TkfYT2KFEgW3ePKEgphig
</commit_message>
<xml_diff>
--- a/Observatii.xlsx
+++ b/Observatii.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t xml:space="preserve">Observații</t>
   </si>
@@ -73,6 +73,18 @@
     <t xml:space="preserve">CONFIRMAT (cardurile mici din listă). Fiecare din cele 8 .collection-item-3 are a.blog-link-block.hide-mobile-landscape → .blog21_featured-item.small-card (desktop) și div.mobile-blog-card.list (mobil), cu același conținut (ex. „10 best 3PL companies in Dallas, TX (2026)”, Locations, 14 Min read).
 Efecte: tot conținutul listei e dublat în HTML (8 titluri, rezumate, imagini, linkuri); se încarcă dublu și la paginarea Finsweet CMS Load. h4 desktop / h6 mobil, alt gol, „Read more” generic; autor gol pe desktop, lipsă pe mobil.
 FIX: păstrează doar .blog21_featured-item.small-card, adaptat la mobile landscape; șterge .mobile-blog-card.list din Collection Item și scoate hide-mobile-landscape de pe .blog-link-block. Verifică apoi CMS Filter și CMS Load.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.saltbox.com/resources/member-stories-overview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wrapper la button cu absolute si z index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMAT, bug vizual. În member-blocks-tablet (9/9 itemi) wrapper-ul butonului are „margin-top margin-medium z-index-1 absolute-positioning”; cardurile au înălțime fixă (~256px), deci la 360px Read more acoperă textul (Bamblu: „through”, Retrovert: „into reality”; Shinery atinge butonul). La 667px nu se suprapune, dar rămâne ~60px gol la textele scurte.
+z-index-1 nu are peste ce să stea (info-link-block e o iconiță mică, ascunsă sub 767px); margin-top nu are efect pe absolut; Read more e înaintea paragrafului (ordine Tab inversă).
+FIX: layout238_item → Flex vertical, fără înălțime fixă; scoate absolute-positioning și z-index-1; clasă proprie pentru wrapper cu margin-top: auto; mută paragraful deasupra butonului.
+Alte probleme: info-link-block cu href="#" și fără aria-label (x9); pe tabletă butonul e opacity:0 până la hover; două Collection List-uri cu itemi diferiți (Fripper's vs Bamblu), 18 Read more în DOM.</t>
   </si>
 </sst>
 </file>
@@ -636,13 +648,19 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="str">
+      <c r="A8" s="5" t="n">
         <f aca="false">IF(B8="","",ROW()-4)</f>
-        <v/>
-      </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="str">

</xml_diff>